<commit_message>
Automacao WhatsApp integrada ao Excel
</commit_message>
<xml_diff>
--- a/CadastroAcevemistas.xlsx
+++ b/CadastroAcevemistas.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8688"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12264" windowHeight="3288"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -24,14 +24,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>ID</t>
   </si>
   <si>
-    <t xml:space="preserve">Nome </t>
-  </si>
-  <si>
     <t>Telefone</t>
   </si>
   <si>
@@ -60,6 +57,21 @@
   </si>
   <si>
     <t>Ativo</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t>Djinane Antonia</t>
+  </si>
+  <si>
+    <t>djinanereisl@gmail.com</t>
+  </si>
+  <si>
+    <t>30.00</t>
+  </si>
+  <si>
+    <t>DataCadastro</t>
   </si>
 </sst>
 </file>
@@ -389,47 +401,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
+      <c r="I1" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>21</v>
@@ -438,21 +454,54 @@
         <v>21968797000</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
         <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
       </c>
       <c r="G2" s="2">
         <v>46190</v>
       </c>
       <c r="H2" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="I2" s="2">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3">
+        <v>14</v>
+      </c>
+      <c r="D3">
+        <v>21966171018</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H3" t="s">
+        <v>10</v>
+      </c>
+      <c r="I3" s="2">
+        <v>46174</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>
+    <hyperlink ref="E3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona envio de WhatsApp para todos os contatos
</commit_message>
<xml_diff>
--- a/CadastroAcevemistas.xlsx
+++ b/CadastroAcevemistas.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>ID</t>
   </si>
@@ -72,6 +72,12 @@
   </si>
   <si>
     <t>DataCadastro</t>
+  </si>
+  <si>
+    <t>Juliana Ramalho</t>
+  </si>
+  <si>
+    <t>20.00</t>
   </si>
 </sst>
 </file>
@@ -401,10 +407,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
@@ -498,6 +504,32 @@
         <v>46174</v>
       </c>
     </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4">
+        <v>24</v>
+      </c>
+      <c r="D4">
+        <v>21974403771</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I4" s="2">
+        <v>46174</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>

</xml_diff>

<commit_message>
Adiciona seleção de imagens e melhorias na automação do WhatsApp
</commit_message>
<xml_diff>
--- a/CadastroAcevemistas.xlsx
+++ b/CadastroAcevemistas.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
     <t>ID</t>
   </si>
@@ -74,10 +74,13 @@
     <t>DataCadastro</t>
   </si>
   <si>
+    <t>Mauriceia</t>
+  </si>
+  <si>
     <t>Juliana Ramalho</t>
   </si>
   <si>
-    <t>20.00</t>
+    <t>Luan Aveiro</t>
   </si>
 </sst>
 </file>
@@ -407,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
@@ -512,13 +515,13 @@
         <v>16</v>
       </c>
       <c r="C4">
-        <v>24</v>
+        <v>141</v>
       </c>
       <c r="D4">
-        <v>21974403771</v>
+        <v>21997984334</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G4" s="2">
         <v>46191</v>
@@ -527,6 +530,58 @@
         <v>10</v>
       </c>
       <c r="I4" s="2">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5">
+        <v>243</v>
+      </c>
+      <c r="D5">
+        <v>21974403771</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H5" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="2">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6">
+        <v>143</v>
+      </c>
+      <c r="D6">
+        <v>21968759702</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I6" s="2">
         <v>46174</v>
       </c>
     </row>

</xml_diff>